<commit_message>
Corregir formatos de la hoja comparativa y agregar utilidades de render
Los estilos se compartian entre celdas, asi que el ultimo formato numerico
aplicado se propagaba a toda la hoja Cambio v3 a v4 y mostraba todo en
dolares. Ahora cada celda recibe una copia de su estilo.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/modelo_capacidad/Modelo_Capacidad_CUADRO_v4.xlsx
+++ b/modelo_capacidad/Modelo_Capacidad_CUADRO_v4.xlsx
@@ -172,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -237,6 +237,7 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -5122,14 +5123,14 @@
           <t>Overlock — capacidad neta (ops/día)</t>
         </is>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="19" t="n">
         <v>1543.6</v>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="25">
         <f>Capacidad!D5</f>
         <v/>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="19">
         <f>C6-B6</f>
         <v/>
       </c>
@@ -5145,14 +5146,14 @@
           <t>Piezas/día (restricción activa)</t>
         </is>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="19" t="n">
         <v>220.514285714286</v>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="25">
         <f>Capacidad!D23</f>
         <v/>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="19">
         <f>C7-B7</f>
         <v/>
       </c>
@@ -5168,14 +5169,14 @@
           <t>Piezas/mes netas de reproceso</t>
         </is>
       </c>
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="30" t="n">
         <v>4233.87428571429</v>
       </c>
-      <c r="C8" s="39">
+      <c r="C8" s="31">
         <f>Capacidad!D26</f>
         <v/>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="30">
         <f>C8-B8</f>
         <v/>
       </c>
@@ -5191,14 +5192,14 @@
           <t>Déficit / superávit — mes regular</t>
         </is>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="33" t="n">
         <v>-325.625714285714</v>
       </c>
-      <c r="C9" s="39">
+      <c r="C9" s="38">
         <f>'Demanda y Deficit'!E5</f>
         <v/>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="33">
         <f>C9-B9</f>
         <v/>
       </c>
@@ -5214,14 +5215,14 @@
           <t>Máquinas a comprar</t>
         </is>
       </c>
-      <c r="B10" s="38" t="n">
+      <c r="B10" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="C10" s="39">
+      <c r="C10" s="31">
         <f>Escenarios!D6</f>
         <v/>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="30">
         <f>C10-B10</f>
         <v/>
       </c>
@@ -5237,14 +5238,14 @@
           <t>Inversión US$</t>
         </is>
       </c>
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="39" t="n">
         <v>20800</v>
       </c>
-      <c r="C11" s="39">
+      <c r="C11" s="40">
         <f>Inversion!H6</f>
         <v/>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="39">
         <f>C11-B11</f>
         <v/>
       </c>
@@ -5271,14 +5272,14 @@
           <t>Overlock — capacidad neta (ops/día)</t>
         </is>
       </c>
-      <c r="B14" s="38" t="n">
+      <c r="B14" s="19" t="n">
         <v>1582.4</v>
       </c>
-      <c r="C14" s="39">
+      <c r="C14" s="25">
         <f>Capacidad!E5</f>
         <v/>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="19">
         <f>C14-B14</f>
         <v/>
       </c>
@@ -5294,14 +5295,14 @@
           <t>Piezas/día (restricción activa)</t>
         </is>
       </c>
-      <c r="B15" s="38" t="n">
+      <c r="B15" s="19" t="n">
         <v>226.057142857143</v>
       </c>
-      <c r="C15" s="39">
+      <c r="C15" s="25">
         <f>Capacidad!E23</f>
         <v/>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="19">
         <f>C15-B15</f>
         <v/>
       </c>
@@ -5317,14 +5318,14 @@
           <t>Piezas/mes netas de reproceso</t>
         </is>
       </c>
-      <c r="B16" s="38" t="n">
+      <c r="B16" s="30" t="n">
         <v>4340.29714285714</v>
       </c>
-      <c r="C16" s="39">
+      <c r="C16" s="31">
         <f>Capacidad!E26</f>
         <v/>
       </c>
-      <c r="D16" s="38">
+      <c r="D16" s="30">
         <f>C16-B16</f>
         <v/>
       </c>
@@ -5340,14 +5341,14 @@
           <t>Déficit / superávit — mes regular</t>
         </is>
       </c>
-      <c r="B17" s="38" t="n">
+      <c r="B17" s="33" t="n">
         <v>-219.202857142856</v>
       </c>
-      <c r="C17" s="39">
+      <c r="C17" s="38">
         <f>'Demanda y Deficit'!F5</f>
         <v/>
       </c>
-      <c r="D17" s="38">
+      <c r="D17" s="33">
         <f>C17-B17</f>
         <v/>
       </c>
@@ -5363,14 +5364,14 @@
           <t>Máquinas a comprar</t>
         </is>
       </c>
-      <c r="B18" s="38" t="n">
+      <c r="B18" s="30" t="n">
         <v>9</v>
       </c>
-      <c r="C18" s="39">
+      <c r="C18" s="31">
         <f>Escenarios!D7</f>
         <v/>
       </c>
-      <c r="D18" s="38">
+      <c r="D18" s="30">
         <f>C18-B18</f>
         <v/>
       </c>
@@ -5386,14 +5387,14 @@
           <t>Inversión US$</t>
         </is>
       </c>
-      <c r="B19" s="38" t="n">
+      <c r="B19" s="39" t="n">
         <v>23800</v>
       </c>
-      <c r="C19" s="39">
+      <c r="C19" s="40">
         <f>Inversion!H7</f>
         <v/>
       </c>
-      <c r="D19" s="38">
+      <c r="D19" s="39">
         <f>C19-B19</f>
         <v/>
       </c>
@@ -5420,14 +5421,14 @@
           <t>Overlock — capacidad neta (ops/día)</t>
         </is>
       </c>
-      <c r="B22" s="38" t="n">
+      <c r="B22" s="19" t="n">
         <v>2001.44</v>
       </c>
-      <c r="C22" s="39">
+      <c r="C22" s="25">
         <f>Capacidad!F5</f>
         <v/>
       </c>
-      <c r="D22" s="38">
+      <c r="D22" s="19">
         <f>C22-B22</f>
         <v/>
       </c>
@@ -5443,14 +5444,14 @@
           <t>Piezas/día (restricción activa)</t>
         </is>
       </c>
-      <c r="B23" s="38" t="n">
+      <c r="B23" s="19" t="n">
         <v>285.92</v>
       </c>
-      <c r="C23" s="39">
+      <c r="C23" s="25">
         <f>Capacidad!F23</f>
         <v/>
       </c>
-      <c r="D23" s="38">
+      <c r="D23" s="19">
         <f>C23-B23</f>
         <v/>
       </c>
@@ -5466,14 +5467,14 @@
           <t>Piezas/mes netas de reproceso</t>
         </is>
       </c>
-      <c r="B24" s="38" t="n">
+      <c r="B24" s="30" t="n">
         <v>5518.256</v>
       </c>
-      <c r="C24" s="39">
+      <c r="C24" s="31">
         <f>Capacidad!F26</f>
         <v/>
       </c>
-      <c r="D24" s="38">
+      <c r="D24" s="30">
         <f>C24-B24</f>
         <v/>
       </c>
@@ -5489,14 +5490,14 @@
           <t>Déficit / superávit — mes regular</t>
         </is>
       </c>
-      <c r="B25" s="38" t="n">
+      <c r="B25" s="33" t="n">
         <v>958.756</v>
       </c>
-      <c r="C25" s="39">
+      <c r="C25" s="38">
         <f>'Demanda y Deficit'!G5</f>
         <v/>
       </c>
-      <c r="D25" s="38">
+      <c r="D25" s="33">
         <f>C25-B25</f>
         <v/>
       </c>
@@ -5512,14 +5513,14 @@
           <t>Máquinas a comprar</t>
         </is>
       </c>
-      <c r="B26" s="38" t="n">
+      <c r="B26" s="30" t="n">
         <v>14</v>
       </c>
-      <c r="C26" s="39">
+      <c r="C26" s="31">
         <f>Escenarios!D8</f>
         <v/>
       </c>
-      <c r="D26" s="38">
+      <c r="D26" s="30">
         <f>C26-B26</f>
         <v/>
       </c>
@@ -5535,14 +5536,14 @@
           <t>Inversión US$</t>
         </is>
       </c>
-      <c r="B27" s="38" t="n">
+      <c r="B27" s="39" t="n">
         <v>34500</v>
       </c>
-      <c r="C27" s="39">
+      <c r="C27" s="40">
         <f>Inversion!H8</f>
         <v/>
       </c>
-      <c r="D27" s="38">
+      <c r="D27" s="39">
         <f>C27-B27</f>
         <v/>
       </c>

</xml_diff>